<commit_message>
fix: admin export now writes to row 6 (not 231+) and un-hides data rows
- _discover_admin_template_mapping: always return best_header_row + 1,
  ignoring hidden staging rows (fixes START_ROW = 231 bug)
- After filling data, ensure written rows have 'hidden' attribute removed
- Cleaned template: removed hidden=1 from all 225 staging rows (6-230)
  so old sample data never leaks into exports
</commit_message>
<xml_diff>
--- a/app/templates/Template_Programacion_Administracion.xlsx
+++ b/app/templates/Template_Programacion_Administracion.xlsx
@@ -696,7 +696,7 @@
         </is>
       </c>
     </row>
-    <row r="6" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="6" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A6" s="6" t="inlineStr">
         <is>
           <t>209</t>
@@ -742,7 +742,7 @@
         </is>
       </c>
     </row>
-    <row r="7" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="7" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A7" s="6" t="inlineStr">
         <is>
           <t>210</t>
@@ -788,7 +788,7 @@
         </is>
       </c>
     </row>
-    <row r="8" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="8" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A8" s="6" t="inlineStr">
         <is>
           <t>211</t>
@@ -834,7 +834,7 @@
         </is>
       </c>
     </row>
-    <row r="9" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="9" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A9" s="6" t="inlineStr">
         <is>
           <t>212</t>
@@ -876,7 +876,7 @@
       </c>
       <c r="L9" s="9" t="n"/>
     </row>
-    <row r="10" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="10" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A10" s="6" t="inlineStr">
         <is>
           <t>213</t>
@@ -922,7 +922,7 @@
         </is>
       </c>
     </row>
-    <row r="11" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="11" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A11" s="6" t="inlineStr">
         <is>
           <t>214</t>
@@ -964,7 +964,7 @@
       </c>
       <c r="L11" s="9" t="n"/>
     </row>
-    <row r="12" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="12" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A12" s="6" t="inlineStr">
         <is>
           <t>215</t>
@@ -1006,7 +1006,7 @@
       </c>
       <c r="L12" s="9" t="n"/>
     </row>
-    <row r="13" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="13" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A13" s="6" t="inlineStr">
         <is>
           <t>216</t>
@@ -1052,7 +1052,7 @@
         </is>
       </c>
     </row>
-    <row r="14" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="14" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A14" s="6" t="inlineStr">
         <is>
           <t>217</t>
@@ -1094,7 +1094,7 @@
       </c>
       <c r="L14" s="9" t="n"/>
     </row>
-    <row r="15" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="15" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A15" s="6" t="inlineStr">
         <is>
           <t>218</t>
@@ -1136,7 +1136,7 @@
       </c>
       <c r="L15" s="9" t="n"/>
     </row>
-    <row r="16" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="16" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A16" s="6" t="inlineStr">
         <is>
           <t>219</t>
@@ -1178,7 +1178,7 @@
       </c>
       <c r="L16" s="9" t="n"/>
     </row>
-    <row r="17" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="17" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A17" s="6" t="inlineStr">
         <is>
           <t>220</t>
@@ -1220,7 +1220,7 @@
       </c>
       <c r="L17" s="9" t="n"/>
     </row>
-    <row r="18" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="18" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A18" s="6" t="inlineStr">
         <is>
           <t>221</t>
@@ -1266,7 +1266,7 @@
         </is>
       </c>
     </row>
-    <row r="19" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="19" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A19" s="6" t="inlineStr">
         <is>
           <t>222</t>
@@ -1308,7 +1308,7 @@
       </c>
       <c r="L19" s="9" t="n"/>
     </row>
-    <row r="20" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="20" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A20" s="6" t="inlineStr">
         <is>
           <t>223</t>
@@ -1342,7 +1342,7 @@
       </c>
       <c r="L20" s="9" t="n"/>
     </row>
-    <row r="21" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="21" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A21" s="6" t="inlineStr">
         <is>
           <t>224</t>
@@ -1388,7 +1388,7 @@
         </is>
       </c>
     </row>
-    <row r="22" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="22" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A22" s="6" t="inlineStr">
         <is>
           <t>225</t>
@@ -1434,7 +1434,7 @@
         </is>
       </c>
     </row>
-    <row r="23" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="23" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A23" s="6" t="inlineStr">
         <is>
           <t>226</t>
@@ -1480,7 +1480,7 @@
         </is>
       </c>
     </row>
-    <row r="24" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="24" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A24" s="6" t="inlineStr">
         <is>
           <t>227</t>
@@ -1526,7 +1526,7 @@
         </is>
       </c>
     </row>
-    <row r="25" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="25" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A25" s="6" t="inlineStr">
         <is>
           <t>228</t>
@@ -1572,7 +1572,7 @@
         </is>
       </c>
     </row>
-    <row r="26" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="26" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A26" s="6" t="inlineStr">
         <is>
           <t>229</t>
@@ -1614,7 +1614,7 @@
       </c>
       <c r="L26" s="9" t="n"/>
     </row>
-    <row r="27" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="27" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A27" s="6" t="inlineStr">
         <is>
           <t>230</t>
@@ -1660,7 +1660,7 @@
         </is>
       </c>
     </row>
-    <row r="28" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="28" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A28" s="6" t="inlineStr">
         <is>
           <t>231</t>
@@ -1702,7 +1702,7 @@
       </c>
       <c r="L28" s="9" t="n"/>
     </row>
-    <row r="29" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="29" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A29" s="6" t="inlineStr">
         <is>
           <t>232</t>
@@ -1736,7 +1736,7 @@
       </c>
       <c r="L29" s="9" t="n"/>
     </row>
-    <row r="30" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="30" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A30" s="6" t="inlineStr">
         <is>
           <t>233</t>
@@ -1778,7 +1778,7 @@
       </c>
       <c r="L30" s="9" t="n"/>
     </row>
-    <row r="31" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="31" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A31" s="6" t="inlineStr">
         <is>
           <t>234</t>
@@ -1820,7 +1820,7 @@
       </c>
       <c r="L31" s="9" t="n"/>
     </row>
-    <row r="32" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="32" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A32" s="6" t="inlineStr">
         <is>
           <t>235</t>
@@ -1862,7 +1862,7 @@
       </c>
       <c r="L32" s="9" t="n"/>
     </row>
-    <row r="33" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="33" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A33" s="6" t="inlineStr">
         <is>
           <t>236</t>
@@ -1908,7 +1908,7 @@
         </is>
       </c>
     </row>
-    <row r="34" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="34" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A34" s="6" t="inlineStr">
         <is>
           <t>237</t>
@@ -1954,7 +1954,7 @@
         </is>
       </c>
     </row>
-    <row r="35" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="35" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A35" s="6" t="inlineStr">
         <is>
           <t>238</t>
@@ -2000,7 +2000,7 @@
         </is>
       </c>
     </row>
-    <row r="36" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="36" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A36" s="6" t="inlineStr">
         <is>
           <t>239</t>
@@ -2046,7 +2046,7 @@
         </is>
       </c>
     </row>
-    <row r="37" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="37" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A37" s="6" t="inlineStr">
         <is>
           <t>240</t>
@@ -2088,7 +2088,7 @@
       </c>
       <c r="L37" s="9" t="n"/>
     </row>
-    <row r="38" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="38" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A38" s="6" t="inlineStr">
         <is>
           <t>241</t>
@@ -2134,7 +2134,7 @@
         </is>
       </c>
     </row>
-    <row r="39" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="39" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A39" s="6" t="inlineStr">
         <is>
           <t>242</t>
@@ -2180,7 +2180,7 @@
         </is>
       </c>
     </row>
-    <row r="40" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="40" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A40" s="6" t="inlineStr">
         <is>
           <t>243</t>
@@ -2226,7 +2226,7 @@
         </is>
       </c>
     </row>
-    <row r="41" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="41" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A41" s="6" t="inlineStr">
         <is>
           <t>244</t>
@@ -2268,7 +2268,7 @@
       </c>
       <c r="L41" s="9" t="n"/>
     </row>
-    <row r="42" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="42" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A42" s="6" t="inlineStr">
         <is>
           <t>245</t>
@@ -2310,7 +2310,7 @@
       </c>
       <c r="L42" s="9" t="n"/>
     </row>
-    <row r="43" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="43" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A43" s="6" t="inlineStr">
         <is>
           <t>246</t>
@@ -2356,7 +2356,7 @@
         </is>
       </c>
     </row>
-    <row r="44" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="44" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A44" s="6" t="inlineStr">
         <is>
           <t>247</t>
@@ -2402,7 +2402,7 @@
         </is>
       </c>
     </row>
-    <row r="45" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="45" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A45" s="6" t="inlineStr">
         <is>
           <t>248</t>
@@ -2448,7 +2448,7 @@
         </is>
       </c>
     </row>
-    <row r="46" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="46" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A46" s="6" t="inlineStr">
         <is>
           <t>249</t>
@@ -2490,7 +2490,7 @@
       </c>
       <c r="L46" s="9" t="n"/>
     </row>
-    <row r="47" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="47" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A47" s="6" t="inlineStr">
         <is>
           <t>250</t>
@@ -2536,7 +2536,7 @@
         </is>
       </c>
     </row>
-    <row r="48" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="48" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A48" s="6" t="inlineStr">
         <is>
           <t>251</t>
@@ -2570,7 +2570,7 @@
       </c>
       <c r="L48" s="9" t="n"/>
     </row>
-    <row r="49" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="49" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A49" s="6" t="inlineStr">
         <is>
           <t>252</t>
@@ -2604,7 +2604,7 @@
       </c>
       <c r="L49" s="9" t="n"/>
     </row>
-    <row r="50" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="50" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A50" s="6" t="inlineStr">
         <is>
           <t>253</t>
@@ -2646,7 +2646,7 @@
       </c>
       <c r="L50" s="9" t="n"/>
     </row>
-    <row r="51" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="51" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A51" s="6" t="inlineStr">
         <is>
           <t>254</t>
@@ -2688,7 +2688,7 @@
       </c>
       <c r="L51" s="9" t="n"/>
     </row>
-    <row r="52" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="52" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A52" s="6" t="inlineStr">
         <is>
           <t>255</t>
@@ -2730,7 +2730,7 @@
       </c>
       <c r="L52" s="9" t="n"/>
     </row>
-    <row r="53" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="53" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A53" s="6" t="inlineStr">
         <is>
           <t>256</t>
@@ -2776,7 +2776,7 @@
         </is>
       </c>
     </row>
-    <row r="54" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="54" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A54" s="6" t="inlineStr">
         <is>
           <t>257</t>
@@ -2822,7 +2822,7 @@
         </is>
       </c>
     </row>
-    <row r="55" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="55" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A55" s="6" t="inlineStr">
         <is>
           <t>258</t>
@@ -2868,7 +2868,7 @@
         </is>
       </c>
     </row>
-    <row r="56" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="56" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A56" s="6" t="inlineStr">
         <is>
           <t>259</t>
@@ -2910,7 +2910,7 @@
       </c>
       <c r="L56" s="9" t="n"/>
     </row>
-    <row r="57" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="57" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A57" s="6" t="inlineStr">
         <is>
           <t>260</t>
@@ -2956,7 +2956,7 @@
         </is>
       </c>
     </row>
-    <row r="58" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="58" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A58" s="6" t="inlineStr">
         <is>
           <t>261</t>
@@ -2998,7 +2998,7 @@
       </c>
       <c r="L58" s="9" t="n"/>
     </row>
-    <row r="59" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="59" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A59" s="6" t="inlineStr">
         <is>
           <t>262</t>
@@ -3040,7 +3040,7 @@
       </c>
       <c r="L59" s="9" t="n"/>
     </row>
-    <row r="60" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="60" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A60" s="6" t="inlineStr">
         <is>
           <t>263</t>
@@ -3086,7 +3086,7 @@
         </is>
       </c>
     </row>
-    <row r="61" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="61" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A61" s="6" t="inlineStr">
         <is>
           <t>264</t>
@@ -3128,7 +3128,7 @@
       </c>
       <c r="L61" s="9" t="n"/>
     </row>
-    <row r="62" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="62" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A62" s="6" t="inlineStr">
         <is>
           <t>265</t>
@@ -3170,7 +3170,7 @@
       </c>
       <c r="L62" s="9" t="n"/>
     </row>
-    <row r="63" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="63" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A63" s="6" t="inlineStr">
         <is>
           <t>266</t>
@@ -3212,7 +3212,7 @@
       </c>
       <c r="L63" s="9" t="n"/>
     </row>
-    <row r="64" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="64" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A64" s="6" t="inlineStr">
         <is>
           <t>267</t>
@@ -3254,7 +3254,7 @@
       </c>
       <c r="L64" s="9" t="n"/>
     </row>
-    <row r="65" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="65" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A65" s="6" t="inlineStr">
         <is>
           <t>268</t>
@@ -3296,7 +3296,7 @@
       </c>
       <c r="L65" s="9" t="n"/>
     </row>
-    <row r="66" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="66" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A66" s="6" t="inlineStr">
         <is>
           <t>269</t>
@@ -3342,7 +3342,7 @@
         </is>
       </c>
     </row>
-    <row r="67" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="67" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A67" s="6" t="inlineStr">
         <is>
           <t>270</t>
@@ -3388,7 +3388,7 @@
         </is>
       </c>
     </row>
-    <row r="68" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="68" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A68" s="6" t="inlineStr">
         <is>
           <t>271</t>
@@ -3430,7 +3430,7 @@
       </c>
       <c r="L68" s="9" t="n"/>
     </row>
-    <row r="69" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="69" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A69" s="6" t="inlineStr">
         <is>
           <t>272</t>
@@ -3476,7 +3476,7 @@
         </is>
       </c>
     </row>
-    <row r="70" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="70" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A70" s="6" t="inlineStr">
         <is>
           <t>273</t>
@@ -3518,7 +3518,7 @@
       </c>
       <c r="L70" s="9" t="n"/>
     </row>
-    <row r="71" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="71" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A71" s="6" t="inlineStr">
         <is>
           <t>274</t>
@@ -3560,7 +3560,7 @@
       </c>
       <c r="L71" s="9" t="n"/>
     </row>
-    <row r="72" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="72" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A72" s="6" t="inlineStr">
         <is>
           <t>275</t>
@@ -3602,7 +3602,7 @@
       </c>
       <c r="L72" s="9" t="n"/>
     </row>
-    <row r="73" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="73" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A73" s="6" t="inlineStr">
         <is>
           <t>276</t>
@@ -3644,7 +3644,7 @@
       </c>
       <c r="L73" s="9" t="n"/>
     </row>
-    <row r="74" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="74" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A74" s="6" t="inlineStr">
         <is>
           <t>277</t>
@@ -3686,7 +3686,7 @@
       </c>
       <c r="L74" s="9" t="n"/>
     </row>
-    <row r="75" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="75" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A75" s="6" t="inlineStr">
         <is>
           <t>278</t>
@@ -3728,7 +3728,7 @@
       </c>
       <c r="L75" s="9" t="n"/>
     </row>
-    <row r="76" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="76" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A76" s="6" t="inlineStr">
         <is>
           <t>279</t>
@@ -3770,7 +3770,7 @@
       </c>
       <c r="L76" s="9" t="n"/>
     </row>
-    <row r="77" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="77" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A77" s="6" t="inlineStr">
         <is>
           <t>280</t>
@@ -3812,7 +3812,7 @@
       </c>
       <c r="L77" s="9" t="n"/>
     </row>
-    <row r="78" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="78" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A78" s="6" t="inlineStr">
         <is>
           <t>281</t>
@@ -3858,7 +3858,7 @@
         </is>
       </c>
     </row>
-    <row r="79" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="79" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A79" s="6" t="inlineStr">
         <is>
           <t>282</t>
@@ -3904,7 +3904,7 @@
         </is>
       </c>
     </row>
-    <row r="80" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="80" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A80" s="6" t="inlineStr">
         <is>
           <t>283</t>
@@ -3946,7 +3946,7 @@
       </c>
       <c r="L80" s="9" t="n"/>
     </row>
-    <row r="81" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="81" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A81" s="6" t="inlineStr">
         <is>
           <t>284</t>
@@ -3988,7 +3988,7 @@
       </c>
       <c r="L81" s="9" t="n"/>
     </row>
-    <row r="82" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="82" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A82" s="6" t="inlineStr">
         <is>
           <t>285</t>
@@ -4034,7 +4034,7 @@
         </is>
       </c>
     </row>
-    <row r="83" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="83" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A83" s="6" t="inlineStr">
         <is>
           <t>286</t>
@@ -4080,7 +4080,7 @@
         </is>
       </c>
     </row>
-    <row r="84" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="84" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A84" s="6" t="inlineStr">
         <is>
           <t>287</t>
@@ -4126,7 +4126,7 @@
         </is>
       </c>
     </row>
-    <row r="85" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="85" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A85" s="6" t="inlineStr">
         <is>
           <t>288</t>
@@ -4168,7 +4168,7 @@
       </c>
       <c r="L85" s="9" t="n"/>
     </row>
-    <row r="86" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="86" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A86" s="6" t="inlineStr">
         <is>
           <t>289</t>
@@ -4210,7 +4210,7 @@
       </c>
       <c r="L86" s="9" t="n"/>
     </row>
-    <row r="87" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="87" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A87" s="6" t="inlineStr">
         <is>
           <t>290</t>
@@ -4256,7 +4256,7 @@
         </is>
       </c>
     </row>
-    <row r="88" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="88" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A88" s="6" t="inlineStr">
         <is>
           <t>291</t>
@@ -4302,7 +4302,7 @@
         </is>
       </c>
     </row>
-    <row r="89" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="89" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A89" s="6" t="inlineStr">
         <is>
           <t>292</t>
@@ -4348,7 +4348,7 @@
         </is>
       </c>
     </row>
-    <row r="90" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="90" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A90" s="6" t="inlineStr">
         <is>
           <t>293</t>
@@ -4390,7 +4390,7 @@
       </c>
       <c r="L90" s="9" t="n"/>
     </row>
-    <row r="91" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="91" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A91" s="6" t="inlineStr">
         <is>
           <t>294</t>
@@ -4432,7 +4432,7 @@
       </c>
       <c r="L91" s="9" t="n"/>
     </row>
-    <row r="92" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="92" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A92" s="6" t="inlineStr">
         <is>
           <t>295</t>
@@ -4478,7 +4478,7 @@
         </is>
       </c>
     </row>
-    <row r="93" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="93" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A93" s="6" t="inlineStr">
         <is>
           <t>296</t>
@@ -4524,7 +4524,7 @@
         </is>
       </c>
     </row>
-    <row r="94" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="94" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A94" s="6" t="inlineStr">
         <is>
           <t>297</t>
@@ -4558,7 +4558,7 @@
       </c>
       <c r="L94" s="9" t="n"/>
     </row>
-    <row r="95" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="95" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A95" s="6" t="inlineStr">
         <is>
           <t>298</t>
@@ -4592,7 +4592,7 @@
       </c>
       <c r="L95" s="9" t="n"/>
     </row>
-    <row r="96" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="96" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A96" s="6" t="inlineStr">
         <is>
           <t>299</t>
@@ -4626,7 +4626,7 @@
       </c>
       <c r="L96" s="9" t="n"/>
     </row>
-    <row r="97" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="97" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A97" s="6" t="inlineStr">
         <is>
           <t>300</t>
@@ -4660,7 +4660,7 @@
       </c>
       <c r="L97" s="9" t="n"/>
     </row>
-    <row r="98" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="98" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A98" s="6" t="inlineStr">
         <is>
           <t>301</t>
@@ -4694,7 +4694,7 @@
       </c>
       <c r="L98" s="9" t="n"/>
     </row>
-    <row r="99" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="99" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A99" s="6" t="inlineStr">
         <is>
           <t>302</t>
@@ -4736,7 +4736,7 @@
       </c>
       <c r="L99" s="9" t="n"/>
     </row>
-    <row r="100" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="100" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A100" s="6" t="inlineStr">
         <is>
           <t>303</t>
@@ -4782,7 +4782,7 @@
         </is>
       </c>
     </row>
-    <row r="101" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="101" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A101" s="6" t="inlineStr">
         <is>
           <t>304</t>
@@ -4828,7 +4828,7 @@
         </is>
       </c>
     </row>
-    <row r="102" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="102" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A102" s="6" t="inlineStr">
         <is>
           <t>305</t>
@@ -4874,7 +4874,7 @@
         </is>
       </c>
     </row>
-    <row r="103" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="103" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A103" s="6" t="inlineStr">
         <is>
           <t>306</t>
@@ -4916,7 +4916,7 @@
       </c>
       <c r="L103" s="9" t="n"/>
     </row>
-    <row r="104" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="104" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A104" s="6" t="inlineStr">
         <is>
           <t>307</t>
@@ -4958,7 +4958,7 @@
       </c>
       <c r="L104" s="9" t="n"/>
     </row>
-    <row r="105" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="105" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A105" s="6" t="inlineStr">
         <is>
           <t>308</t>
@@ -5000,7 +5000,7 @@
       </c>
       <c r="L105" s="9" t="n"/>
     </row>
-    <row r="106" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="106" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A106" s="6" t="inlineStr">
         <is>
           <t>309</t>
@@ -5046,7 +5046,7 @@
         </is>
       </c>
     </row>
-    <row r="107" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="107" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A107" s="6" t="inlineStr">
         <is>
           <t>310</t>
@@ -5088,7 +5088,7 @@
       </c>
       <c r="L107" s="9" t="n"/>
     </row>
-    <row r="108" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="108" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A108" s="6" t="inlineStr">
         <is>
           <t>311</t>
@@ -5130,7 +5130,7 @@
       </c>
       <c r="L108" s="9" t="n"/>
     </row>
-    <row r="109" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="109" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A109" s="6" t="inlineStr">
         <is>
           <t>312</t>
@@ -5172,7 +5172,7 @@
       </c>
       <c r="L109" s="9" t="n"/>
     </row>
-    <row r="110" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="110" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A110" s="6" t="inlineStr">
         <is>
           <t>313</t>
@@ -5214,7 +5214,7 @@
       </c>
       <c r="L110" s="9" t="n"/>
     </row>
-    <row r="111" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="111" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A111" s="6" t="inlineStr">
         <is>
           <t>314</t>
@@ -5260,7 +5260,7 @@
         </is>
       </c>
     </row>
-    <row r="112" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="112" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A112" s="6" t="inlineStr">
         <is>
           <t>315</t>
@@ -5298,7 +5298,7 @@
         </is>
       </c>
     </row>
-    <row r="113" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="113" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A113" s="6" t="inlineStr">
         <is>
           <t>316</t>
@@ -5344,7 +5344,7 @@
         </is>
       </c>
     </row>
-    <row r="114" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="114" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A114" s="6" t="inlineStr">
         <is>
           <t>317</t>
@@ -5386,7 +5386,7 @@
       </c>
       <c r="L114" s="9" t="n"/>
     </row>
-    <row r="115" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="115" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A115" s="6" t="inlineStr">
         <is>
           <t>318</t>
@@ -5428,7 +5428,7 @@
         </is>
       </c>
     </row>
-    <row r="116" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="116" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A116" s="6" t="inlineStr">
         <is>
           <t>319</t>
@@ -5474,7 +5474,7 @@
         </is>
       </c>
     </row>
-    <row r="117" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="117" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A117" s="6" t="inlineStr">
         <is>
           <t>320</t>
@@ -5516,7 +5516,7 @@
       </c>
       <c r="L117" s="9" t="n"/>
     </row>
-    <row r="118" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="118" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A118" s="6" t="inlineStr">
         <is>
           <t>321</t>
@@ -5562,7 +5562,7 @@
         </is>
       </c>
     </row>
-    <row r="119" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="119" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A119" s="6" t="inlineStr">
         <is>
           <t>322</t>
@@ -5604,7 +5604,7 @@
       </c>
       <c r="L119" s="9" t="n"/>
     </row>
-    <row r="120" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="120" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A120" s="6" t="inlineStr">
         <is>
           <t>323</t>
@@ -5646,7 +5646,7 @@
       </c>
       <c r="L120" s="9" t="n"/>
     </row>
-    <row r="121" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="121" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A121" s="6" t="inlineStr">
         <is>
           <t>324</t>
@@ -5688,7 +5688,7 @@
       </c>
       <c r="L121" s="9" t="n"/>
     </row>
-    <row r="122" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="122" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A122" s="6" t="inlineStr">
         <is>
           <t>325</t>
@@ -5734,7 +5734,7 @@
         </is>
       </c>
     </row>
-    <row r="123" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="123" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A123" s="6" t="inlineStr">
         <is>
           <t>326</t>
@@ -5776,7 +5776,7 @@
         </is>
       </c>
     </row>
-    <row r="124" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="124" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A124" s="6" t="inlineStr">
         <is>
           <t>327</t>
@@ -5818,7 +5818,7 @@
       </c>
       <c r="L124" s="9" t="n"/>
     </row>
-    <row r="125" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="125" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A125" s="6" t="inlineStr">
         <is>
           <t>328</t>
@@ -5856,7 +5856,7 @@
         </is>
       </c>
     </row>
-    <row r="126" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="126" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A126" s="6" t="inlineStr">
         <is>
           <t>329</t>
@@ -5898,7 +5898,7 @@
       </c>
       <c r="L126" s="9" t="n"/>
     </row>
-    <row r="127" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="127" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A127" s="6" t="inlineStr">
         <is>
           <t>330</t>
@@ -5944,7 +5944,7 @@
         </is>
       </c>
     </row>
-    <row r="128" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="128" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A128" s="6" t="inlineStr">
         <is>
           <t>331</t>
@@ -5986,7 +5986,7 @@
       </c>
       <c r="L128" s="9" t="n"/>
     </row>
-    <row r="129" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="129" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A129" s="6" t="inlineStr">
         <is>
           <t>332</t>
@@ -6032,7 +6032,7 @@
         </is>
       </c>
     </row>
-    <row r="130" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="130" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A130" s="6" t="inlineStr">
         <is>
           <t>333</t>
@@ -6074,7 +6074,7 @@
         </is>
       </c>
     </row>
-    <row r="131" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="131" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A131" s="6" t="inlineStr">
         <is>
           <t>334</t>
@@ -6120,7 +6120,7 @@
         </is>
       </c>
     </row>
-    <row r="132" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="132" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A132" s="6" t="inlineStr">
         <is>
           <t>335</t>
@@ -6166,7 +6166,7 @@
         </is>
       </c>
     </row>
-    <row r="133" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="133" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A133" s="6" t="inlineStr">
         <is>
           <t>336</t>
@@ -6208,7 +6208,7 @@
       </c>
       <c r="L133" s="9" t="n"/>
     </row>
-    <row r="134" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="134" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A134" s="6" t="inlineStr">
         <is>
           <t>337</t>
@@ -6242,7 +6242,7 @@
       </c>
       <c r="L134" s="9" t="n"/>
     </row>
-    <row r="135" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="135" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A135" s="6" t="inlineStr">
         <is>
           <t>338</t>
@@ -6284,7 +6284,7 @@
       </c>
       <c r="L135" s="9" t="n"/>
     </row>
-    <row r="136" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="136" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A136" s="6" t="inlineStr">
         <is>
           <t>339</t>
@@ -6326,7 +6326,7 @@
       </c>
       <c r="L136" s="9" t="n"/>
     </row>
-    <row r="137" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="137" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A137" s="6" t="inlineStr">
         <is>
           <t>340</t>
@@ -6368,7 +6368,7 @@
       </c>
       <c r="L137" s="9" t="n"/>
     </row>
-    <row r="138" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="138" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A138" s="6" t="inlineStr">
         <is>
           <t>341</t>
@@ -6414,7 +6414,7 @@
         </is>
       </c>
     </row>
-    <row r="139" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="139" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A139" s="6" t="inlineStr">
         <is>
           <t>342</t>
@@ -6456,7 +6456,7 @@
         </is>
       </c>
     </row>
-    <row r="140" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="140" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A140" s="6" t="inlineStr">
         <is>
           <t>343</t>
@@ -6498,7 +6498,7 @@
       </c>
       <c r="L140" s="9" t="n"/>
     </row>
-    <row r="141" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="141" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A141" s="6" t="inlineStr">
         <is>
           <t>344</t>
@@ -6544,7 +6544,7 @@
         </is>
       </c>
     </row>
-    <row r="142" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="142" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A142" s="6" t="inlineStr">
         <is>
           <t>345</t>
@@ -6586,7 +6586,7 @@
       </c>
       <c r="L142" s="9" t="n"/>
     </row>
-    <row r="143" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="143" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A143" s="6" t="inlineStr">
         <is>
           <t>346</t>
@@ -6628,7 +6628,7 @@
       </c>
       <c r="L143" s="9" t="n"/>
     </row>
-    <row r="144" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="144" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A144" s="6" t="inlineStr">
         <is>
           <t>347</t>
@@ -6662,7 +6662,7 @@
       </c>
       <c r="L144" s="9" t="n"/>
     </row>
-    <row r="145" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="145" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A145" s="6" t="inlineStr">
         <is>
           <t>348</t>
@@ -6696,7 +6696,7 @@
       </c>
       <c r="L145" s="9" t="n"/>
     </row>
-    <row r="146" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="146" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A146" s="6" t="inlineStr">
         <is>
           <t>349</t>
@@ -6738,7 +6738,7 @@
       </c>
       <c r="L146" s="9" t="n"/>
     </row>
-    <row r="147" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="147" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A147" s="6" t="inlineStr">
         <is>
           <t>350</t>
@@ -6784,7 +6784,7 @@
         </is>
       </c>
     </row>
-    <row r="148" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="148" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A148" s="6" t="inlineStr">
         <is>
           <t>351</t>
@@ -6826,7 +6826,7 @@
         </is>
       </c>
     </row>
-    <row r="149" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="149" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A149" s="6" t="inlineStr">
         <is>
           <t>352</t>
@@ -6868,7 +6868,7 @@
       </c>
       <c r="L149" s="9" t="n"/>
     </row>
-    <row r="150" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="150" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A150" s="6" t="inlineStr">
         <is>
           <t>353</t>
@@ -6914,7 +6914,7 @@
         </is>
       </c>
     </row>
-    <row r="151" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="151" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A151" s="6" t="inlineStr">
         <is>
           <t>354</t>
@@ -6956,7 +6956,7 @@
       </c>
       <c r="L151" s="9" t="n"/>
     </row>
-    <row r="152" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="152" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A152" s="6" t="inlineStr">
         <is>
           <t>355</t>
@@ -6990,7 +6990,7 @@
       </c>
       <c r="L152" s="9" t="n"/>
     </row>
-    <row r="153" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="153" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A153" s="6" t="inlineStr">
         <is>
           <t>356</t>
@@ -7024,7 +7024,7 @@
       </c>
       <c r="L153" s="9" t="n"/>
     </row>
-    <row r="154" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="154" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A154" s="6" t="inlineStr">
         <is>
           <t>357</t>
@@ -7058,7 +7058,7 @@
       </c>
       <c r="L154" s="9" t="n"/>
     </row>
-    <row r="155" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="155" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A155" s="6" t="inlineStr">
         <is>
           <t>358</t>
@@ -7100,7 +7100,7 @@
       </c>
       <c r="L155" s="9" t="n"/>
     </row>
-    <row r="156" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="156" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A156" s="6" t="inlineStr">
         <is>
           <t>359</t>
@@ -7142,7 +7142,7 @@
       </c>
       <c r="L156" s="9" t="n"/>
     </row>
-    <row r="157" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="157" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A157" s="6" t="inlineStr">
         <is>
           <t>360</t>
@@ -7180,7 +7180,7 @@
         </is>
       </c>
     </row>
-    <row r="158" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="158" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A158" s="6" t="inlineStr">
         <is>
           <t>361</t>
@@ -7226,7 +7226,7 @@
         </is>
       </c>
     </row>
-    <row r="159" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="159" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A159" s="6" t="inlineStr">
         <is>
           <t>362</t>
@@ -7268,7 +7268,7 @@
         </is>
       </c>
     </row>
-    <row r="160" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="160" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A160" s="6" t="inlineStr">
         <is>
           <t>363</t>
@@ -7310,7 +7310,7 @@
       </c>
       <c r="L160" s="9" t="n"/>
     </row>
-    <row r="161" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="161" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A161" s="6" t="inlineStr">
         <is>
           <t>364</t>
@@ -7356,7 +7356,7 @@
         </is>
       </c>
     </row>
-    <row r="162" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="162" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A162" s="6" t="inlineStr">
         <is>
           <t>365</t>
@@ -7398,7 +7398,7 @@
       </c>
       <c r="L162" s="9" t="n"/>
     </row>
-    <row r="163" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="163" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A163" s="6" t="inlineStr">
         <is>
           <t>366</t>
@@ -7440,7 +7440,7 @@
       </c>
       <c r="L163" s="9" t="n"/>
     </row>
-    <row r="164" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="164" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A164" s="6" t="inlineStr">
         <is>
           <t>367</t>
@@ -7478,7 +7478,7 @@
         </is>
       </c>
     </row>
-    <row r="165" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="165" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A165" s="6" t="inlineStr">
         <is>
           <t>368</t>
@@ -7524,7 +7524,7 @@
         </is>
       </c>
     </row>
-    <row r="166" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="166" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A166" s="6" t="inlineStr">
         <is>
           <t>369</t>
@@ -7566,7 +7566,7 @@
         </is>
       </c>
     </row>
-    <row r="167" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="167" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A167" s="6" t="inlineStr">
         <is>
           <t>370</t>
@@ -7608,7 +7608,7 @@
       </c>
       <c r="L167" s="9" t="n"/>
     </row>
-    <row r="168" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="168" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A168" s="6" t="inlineStr">
         <is>
           <t>371</t>
@@ -7650,7 +7650,7 @@
       </c>
       <c r="L168" s="9" t="n"/>
     </row>
-    <row r="169" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="169" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A169" s="6" t="inlineStr">
         <is>
           <t>372</t>
@@ -7696,7 +7696,7 @@
         </is>
       </c>
     </row>
-    <row r="170" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="170" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A170" s="6" t="inlineStr">
         <is>
           <t>373</t>
@@ -7742,7 +7742,7 @@
         </is>
       </c>
     </row>
-    <row r="171" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="171" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A171" s="6" t="inlineStr">
         <is>
           <t>374</t>
@@ -7780,7 +7780,7 @@
         </is>
       </c>
     </row>
-    <row r="172" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="172" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A172" s="6" t="inlineStr">
         <is>
           <t>375</t>
@@ -7826,7 +7826,7 @@
         </is>
       </c>
     </row>
-    <row r="173" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="173" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A173" s="6" t="inlineStr">
         <is>
           <t>376</t>
@@ -7872,7 +7872,7 @@
         </is>
       </c>
     </row>
-    <row r="174" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="174" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A174" s="6" t="inlineStr">
         <is>
           <t>377</t>
@@ -7914,7 +7914,7 @@
         </is>
       </c>
     </row>
-    <row r="175" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="175" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A175" s="6" t="inlineStr">
         <is>
           <t>378</t>
@@ -7956,7 +7956,7 @@
       </c>
       <c r="L175" s="9" t="n"/>
     </row>
-    <row r="176" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="176" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A176" s="6" t="inlineStr">
         <is>
           <t>379</t>
@@ -7990,7 +7990,7 @@
       </c>
       <c r="L176" s="9" t="n"/>
     </row>
-    <row r="177" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="177" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A177" s="6" t="inlineStr">
         <is>
           <t>380</t>
@@ -8024,7 +8024,7 @@
       </c>
       <c r="L177" s="9" t="n"/>
     </row>
-    <row r="178" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="178" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A178" s="6" t="inlineStr">
         <is>
           <t>381</t>
@@ -8066,7 +8066,7 @@
       </c>
       <c r="L178" s="9" t="n"/>
     </row>
-    <row r="179" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="179" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A179" s="6" t="inlineStr">
         <is>
           <t>382</t>
@@ -8108,7 +8108,7 @@
       </c>
       <c r="L179" s="9" t="n"/>
     </row>
-    <row r="180" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="180" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A180" s="6" t="inlineStr">
         <is>
           <t>383</t>
@@ -8150,7 +8150,7 @@
       </c>
       <c r="L180" s="9" t="n"/>
     </row>
-    <row r="181" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="181" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A181" s="6" t="inlineStr">
         <is>
           <t>384</t>
@@ -8192,7 +8192,7 @@
       </c>
       <c r="L181" s="9" t="n"/>
     </row>
-    <row r="182" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="182" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A182" s="6" t="inlineStr">
         <is>
           <t>385</t>
@@ -8234,7 +8234,7 @@
       </c>
       <c r="L182" s="9" t="n"/>
     </row>
-    <row r="183" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="183" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A183" s="6" t="inlineStr">
         <is>
           <t>386</t>
@@ -8276,7 +8276,7 @@
       </c>
       <c r="L183" s="9" t="n"/>
     </row>
-    <row r="184" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="184" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A184" s="6" t="inlineStr">
         <is>
           <t>387</t>
@@ -8322,7 +8322,7 @@
         </is>
       </c>
     </row>
-    <row r="185" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="185" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A185" s="6" t="inlineStr">
         <is>
           <t>388</t>
@@ -8364,7 +8364,7 @@
       </c>
       <c r="L185" s="9" t="n"/>
     </row>
-    <row r="186" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="186" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A186" s="6" t="inlineStr">
         <is>
           <t>389</t>
@@ -8406,7 +8406,7 @@
       </c>
       <c r="L186" s="9" t="n"/>
     </row>
-    <row r="187" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="187" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A187" s="6" t="inlineStr">
         <is>
           <t>390</t>
@@ -8440,7 +8440,7 @@
       </c>
       <c r="L187" s="9" t="n"/>
     </row>
-    <row r="188" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="188" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A188" s="6" t="inlineStr">
         <is>
           <t>391</t>
@@ -8482,7 +8482,7 @@
       </c>
       <c r="L188" s="9" t="n"/>
     </row>
-    <row r="189" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="189" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A189" s="6" t="inlineStr">
         <is>
           <t>392</t>
@@ -8524,7 +8524,7 @@
       </c>
       <c r="L189" s="9" t="n"/>
     </row>
-    <row r="190" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="190" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A190" s="6" t="inlineStr">
         <is>
           <t>393</t>
@@ -8566,7 +8566,7 @@
       </c>
       <c r="L190" s="9" t="n"/>
     </row>
-    <row r="191" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="191" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A191" s="6" t="inlineStr">
         <is>
           <t>394</t>
@@ -8608,7 +8608,7 @@
       </c>
       <c r="L191" s="9" t="n"/>
     </row>
-    <row r="192" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="192" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A192" s="6" t="inlineStr">
         <is>
           <t>395</t>
@@ -8654,7 +8654,7 @@
         </is>
       </c>
     </row>
-    <row r="193" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="193" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A193" s="6" t="inlineStr">
         <is>
           <t>396</t>
@@ -8696,7 +8696,7 @@
       </c>
       <c r="L193" s="9" t="n"/>
     </row>
-    <row r="194" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="194" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A194" s="6" t="inlineStr">
         <is>
           <t>397</t>
@@ -8738,7 +8738,7 @@
       </c>
       <c r="L194" s="9" t="n"/>
     </row>
-    <row r="195" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="195" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A195" s="6" t="inlineStr">
         <is>
           <t>398</t>
@@ -8784,7 +8784,7 @@
         </is>
       </c>
     </row>
-    <row r="196" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="196" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A196" s="6" t="inlineStr">
         <is>
           <t>399</t>
@@ -8826,7 +8826,7 @@
       </c>
       <c r="L196" s="9" t="n"/>
     </row>
-    <row r="197" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="197" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A197" s="6" t="inlineStr">
         <is>
           <t>400</t>
@@ -8868,7 +8868,7 @@
       </c>
       <c r="L197" s="9" t="n"/>
     </row>
-    <row r="198" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="198" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A198" s="6" t="inlineStr">
         <is>
           <t>401</t>
@@ -8910,7 +8910,7 @@
       </c>
       <c r="L198" s="9" t="n"/>
     </row>
-    <row r="199" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="199" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A199" s="6" t="inlineStr">
         <is>
           <t>402</t>
@@ -8948,7 +8948,7 @@
         </is>
       </c>
     </row>
-    <row r="200" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="200" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A200" s="6" t="inlineStr">
         <is>
           <t>403</t>
@@ -8990,7 +8990,7 @@
       </c>
       <c r="L200" s="9" t="n"/>
     </row>
-    <row r="201" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="201" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A201" s="6" t="inlineStr">
         <is>
           <t>404</t>
@@ -9032,7 +9032,7 @@
       </c>
       <c r="L201" s="9" t="n"/>
     </row>
-    <row r="202" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="202" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A202" s="6" t="inlineStr">
         <is>
           <t>405</t>
@@ -9078,7 +9078,7 @@
         </is>
       </c>
     </row>
-    <row r="203" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="203" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A203" s="6" t="inlineStr">
         <is>
           <t>406</t>
@@ -9120,7 +9120,7 @@
       </c>
       <c r="L203" s="9" t="n"/>
     </row>
-    <row r="204" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="204" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A204" s="6" t="inlineStr">
         <is>
           <t>407</t>
@@ -9162,7 +9162,7 @@
         </is>
       </c>
     </row>
-    <row r="205" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="205" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A205" s="6" t="inlineStr">
         <is>
           <t>408</t>
@@ -9204,7 +9204,7 @@
       </c>
       <c r="L205" s="9" t="n"/>
     </row>
-    <row r="206" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="206" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A206" s="6" t="inlineStr">
         <is>
           <t>409</t>
@@ -9246,7 +9246,7 @@
       </c>
       <c r="L206" s="9" t="n"/>
     </row>
-    <row r="207" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="207" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A207" s="6" t="inlineStr">
         <is>
           <t>410</t>
@@ -9288,7 +9288,7 @@
       </c>
       <c r="L207" s="9" t="n"/>
     </row>
-    <row r="208" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="208" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A208" s="6" t="inlineStr">
         <is>
           <t>411</t>
@@ -9330,7 +9330,7 @@
       </c>
       <c r="L208" s="9" t="n"/>
     </row>
-    <row r="209" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="209" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A209" s="6" t="inlineStr">
         <is>
           <t>412</t>
@@ -9372,7 +9372,7 @@
       </c>
       <c r="L209" s="9" t="n"/>
     </row>
-    <row r="210" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="210" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A210" s="6" t="inlineStr">
         <is>
           <t>413</t>
@@ -9414,7 +9414,7 @@
       </c>
       <c r="L210" s="9" t="n"/>
     </row>
-    <row r="211" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="211" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A211" s="6" t="inlineStr">
         <is>
           <t>414</t>
@@ -9460,7 +9460,7 @@
         </is>
       </c>
     </row>
-    <row r="212" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="212" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A212" s="6" t="inlineStr">
         <is>
           <t>415</t>
@@ -9502,7 +9502,7 @@
       </c>
       <c r="L212" s="9" t="n"/>
     </row>
-    <row r="213" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="213" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A213" s="6" t="inlineStr">
         <is>
           <t>416</t>
@@ -9540,7 +9540,7 @@
         </is>
       </c>
     </row>
-    <row r="214" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="214" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A214" s="6" t="inlineStr">
         <is>
           <t>417</t>
@@ -9582,7 +9582,7 @@
       </c>
       <c r="L214" s="9" t="n"/>
     </row>
-    <row r="215" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="215" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A215" s="6" t="inlineStr">
         <is>
           <t>418</t>
@@ -9624,7 +9624,7 @@
       </c>
       <c r="L215" s="9" t="n"/>
     </row>
-    <row r="216" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="216" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A216" s="6" t="inlineStr">
         <is>
           <t>419</t>
@@ -9666,7 +9666,7 @@
       </c>
       <c r="L216" s="9" t="n"/>
     </row>
-    <row r="217" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="217" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A217" s="6" t="inlineStr">
         <is>
           <t>420</t>
@@ -9704,7 +9704,7 @@
         </is>
       </c>
     </row>
-    <row r="218" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="218" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A218" s="6" t="inlineStr">
         <is>
           <t>421</t>
@@ -9738,7 +9738,7 @@
       </c>
       <c r="L218" s="9" t="n"/>
     </row>
-    <row r="219" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="219" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A219" s="6" t="inlineStr">
         <is>
           <t>422</t>
@@ -9772,7 +9772,7 @@
       </c>
       <c r="L219" s="9" t="n"/>
     </row>
-    <row r="220" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="220" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A220" s="6" t="inlineStr">
         <is>
           <t>423</t>
@@ -9806,7 +9806,7 @@
       </c>
       <c r="L220" s="9" t="n"/>
     </row>
-    <row r="221" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="221" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A221" s="6" t="inlineStr">
         <is>
           <t>424</t>
@@ -9848,7 +9848,7 @@
       </c>
       <c r="L221" s="9" t="n"/>
     </row>
-    <row r="222" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="222" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A222" s="6" t="inlineStr">
         <is>
           <t>425</t>
@@ -9890,7 +9890,7 @@
       </c>
       <c r="L222" s="9" t="n"/>
     </row>
-    <row r="223" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="223" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A223" s="6" t="inlineStr">
         <is>
           <t>426</t>
@@ -9932,7 +9932,7 @@
         </is>
       </c>
     </row>
-    <row r="224" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="224" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A224" s="6" t="inlineStr">
         <is>
           <t>427</t>
@@ -9978,7 +9978,7 @@
         </is>
       </c>
     </row>
-    <row r="225" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="225" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A225" s="6" t="inlineStr">
         <is>
           <t>428</t>
@@ -10020,7 +10020,7 @@
       </c>
       <c r="L225" s="9" t="n"/>
     </row>
-    <row r="226" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="226" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A226" s="6" t="inlineStr">
         <is>
           <t>429</t>
@@ -10062,7 +10062,7 @@
       </c>
       <c r="L226" s="9" t="n"/>
     </row>
-    <row r="227" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="227" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A227" s="6" t="inlineStr">
         <is>
           <t>430</t>
@@ -10104,7 +10104,7 @@
         </is>
       </c>
     </row>
-    <row r="228" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="228" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A228" s="6" t="inlineStr">
         <is>
           <t>431</t>
@@ -10142,7 +10142,7 @@
         </is>
       </c>
     </row>
-    <row r="229" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="229" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A229" s="6" t="inlineStr">
         <is>
           <t>432</t>
@@ -10184,7 +10184,7 @@
       </c>
       <c r="L229" s="9" t="n"/>
     </row>
-    <row r="230" hidden="1" ht="18" customFormat="1" customHeight="1" s="4">
+    <row r="230" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="A230" s="6" t="inlineStr">
         <is>
           <t>433</t>

</xml_diff>